<commit_message>
import excel form 1
</commit_message>
<xml_diff>
--- a/scripts/_smoke-template.xlsx
+++ b/scripts/_smoke-template.xlsx
@@ -330,12 +330,447 @@
         </r>
       </text>
     </comment>
+    <comment ref="P2" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">Type of Cover.Own Vehicle Damage Cover? (when Third Party Only)
+</t>
+        </r>
+        <r>
+          <t xml:space="preserve">Column id: policyinfo.typeOfCover__o_tpo_sc0
+</t>
+        </r>
+        <r>
+          <t xml:space="preserve">Type: boolean
+</t>
+        </r>
+        <r>
+          <t xml:space="preserve">CONDITIONAL — only fill this column when "Type of Cover" is set to "Third Party Only" (value: tpo).
+Filling it when the parent has any other value will FAIL the row.
+</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="Q2" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">Type of Cover.Own Vehicle Damage Cover?.Estimate Value (when Third Party Only / yes)
+</t>
+        </r>
+        <r>
+          <t xml:space="preserve">Column id: policyinfo.typeOfCover__o_tpo_sc0__y_bc0
+</t>
+        </r>
+        <r>
+          <t xml:space="preserve">Type: currency
+</t>
+        </r>
+        <r>
+          <t xml:space="preserve">CONDITIONAL (3-level) — only fill this column when:
+  1. "Type of Cover" = "Third Party Only" (value: tpo), AND
+  2. "Own Vehicle Damage Cover?" is set to yes / true.
+Filling it when either parent is out of sync will fail the row.
+</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="R2" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">Make
+</t>
+        </r>
+        <r>
+          <t xml:space="preserve">Column id: vehicleinfo.make
+</t>
+        </r>
+        <r>
+          <t xml:space="preserve">Type: select
+</t>
+        </r>
+        <r>
+          <t xml:space="preserve">Required
+</t>
+        </r>
+        <r>
+          <t xml:space="preserve">
+Allowed: toyota, bmw, honda</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="S2" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">Make.Model
+</t>
+        </r>
+        <r>
+          <t xml:space="preserve">Column id: vehicleinfo.make__sc0_model
+</t>
+        </r>
+        <r>
+          <t xml:space="preserve">Type: select
+</t>
+        </r>
+        <r>
+          <t xml:space="preserve">CONDITIONAL — depends on "Make".
+Allowed values change based on the chosen "Make" (3 parent options use this field).
+No in-cell dropdown because the valid value list differs per row. Make sure your value matches what the wizard would accept.
+</t>
+        </r>
+        <r>
+          <t xml:space="preserve">
+Examples by Make:
+  • toyota: corolla, camry
+  • bmw: x3, x5
+  • honda: civic, accord
+</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="T2" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">Drivers #1 Name
+</t>
+        </r>
+        <r>
+          <t xml:space="preserve">Column id: vehicleinfo.drivers__r1_name
+</t>
+        </r>
+        <r>
+          <t xml:space="preserve">Type: text
+</t>
+        </r>
+        <r>
+          <t xml:space="preserve">REPEATABLE — slot #1 of 4 for "Drivers" (Driver).
+Fill slots IN ORDER: slot #1 first, then #2, etc. A gap (e.g. #1 empty but #2 filled) will FAIL the row.
+up to 4 items configured (template provides 4 slots). at least 1 item(s) required.
+Required within filled slot.
+</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="U2" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">Drivers #1 Age
+</t>
+        </r>
+        <r>
+          <t xml:space="preserve">Column id: vehicleinfo.drivers__r1_age
+</t>
+        </r>
+        <r>
+          <t xml:space="preserve">Type: number
+</t>
+        </r>
+        <r>
+          <t xml:space="preserve">REPEATABLE — slot #1 of 4 for "Drivers" (Driver).
+Fill slots IN ORDER: slot #1 first, then #2, etc. A gap (e.g. #1 empty but #2 filled) will FAIL the row.
+up to 4 items configured (template provides 4 slots). at least 1 item(s) required.
+</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="V2" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">Drivers #2 Name
+</t>
+        </r>
+        <r>
+          <t xml:space="preserve">Column id: vehicleinfo.drivers__r2_name
+</t>
+        </r>
+        <r>
+          <t xml:space="preserve">Type: text
+</t>
+        </r>
+        <r>
+          <t xml:space="preserve">REPEATABLE — slot #2 of 4 for "Drivers" (Driver).
+Fill slots IN ORDER: slot #1 first, then #2, etc. A gap (e.g. #1 empty but #2 filled) will FAIL the row.
+up to 4 items configured (template provides 4 slots). at least 1 item(s) required.
+Required within filled slot.
+</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="W2" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">Drivers #2 Age
+</t>
+        </r>
+        <r>
+          <t xml:space="preserve">Column id: vehicleinfo.drivers__r2_age
+</t>
+        </r>
+        <r>
+          <t xml:space="preserve">Type: number
+</t>
+        </r>
+        <r>
+          <t xml:space="preserve">REPEATABLE — slot #2 of 4 for "Drivers" (Driver).
+Fill slots IN ORDER: slot #1 first, then #2, etc. A gap (e.g. #1 empty but #2 filled) will FAIL the row.
+up to 4 items configured (template provides 4 slots). at least 1 item(s) required.
+</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="X2" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">Drivers #3 Name
+</t>
+        </r>
+        <r>
+          <t xml:space="preserve">Column id: vehicleinfo.drivers__r3_name
+</t>
+        </r>
+        <r>
+          <t xml:space="preserve">Type: text
+</t>
+        </r>
+        <r>
+          <t xml:space="preserve">REPEATABLE — slot #3 of 4 for "Drivers" (Driver).
+Fill slots IN ORDER: slot #1 first, then #2, etc. A gap (e.g. #1 empty but #2 filled) will FAIL the row.
+up to 4 items configured (template provides 4 slots). at least 1 item(s) required.
+Required within filled slot.
+</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="Y2" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">Drivers #3 Age
+</t>
+        </r>
+        <r>
+          <t xml:space="preserve">Column id: vehicleinfo.drivers__r3_age
+</t>
+        </r>
+        <r>
+          <t xml:space="preserve">Type: number
+</t>
+        </r>
+        <r>
+          <t xml:space="preserve">REPEATABLE — slot #3 of 4 for "Drivers" (Driver).
+Fill slots IN ORDER: slot #1 first, then #2, etc. A gap (e.g. #1 empty but #2 filled) will FAIL the row.
+up to 4 items configured (template provides 4 slots). at least 1 item(s) required.
+</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="Z2" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">Drivers #4 Name
+</t>
+        </r>
+        <r>
+          <t xml:space="preserve">Column id: vehicleinfo.drivers__r4_name
+</t>
+        </r>
+        <r>
+          <t xml:space="preserve">Type: text
+</t>
+        </r>
+        <r>
+          <t xml:space="preserve">REPEATABLE — slot #4 of 4 for "Drivers" (Driver).
+Fill slots IN ORDER: slot #1 first, then #2, etc. A gap (e.g. #1 empty but #2 filled) will FAIL the row.
+up to 4 items configured (template provides 4 slots). at least 1 item(s) required.
+Required within filled slot.
+</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AA2" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">Drivers #4 Age
+</t>
+        </r>
+        <r>
+          <t xml:space="preserve">Column id: vehicleinfo.drivers__r4_age
+</t>
+        </r>
+        <r>
+          <t xml:space="preserve">Type: number
+</t>
+        </r>
+        <r>
+          <t xml:space="preserve">REPEATABLE — slot #4 of 4 for "Drivers" (Driver).
+Fill slots IN ORDER: slot #1 first, then #2, etc. A gap (e.g. #1 empty but #2 filled) will FAIL the row.
+up to 4 items configured (template provides 4 slots). at least 1 item(s) required.
+</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AB2" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">Add more drivers?
+</t>
+        </r>
+        <r>
+          <t xml:space="preserve">Column id: extras.moreDriver
+</t>
+        </r>
+        <r>
+          <t xml:space="preserve">Type: boolean
+</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AC2" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">Add more drivers?.Driver Information #1 Last Name (yes)
+</t>
+        </r>
+        <r>
+          <t xml:space="preserve">Column id: extras.moreDriver__y_c0_r1_lastName
+</t>
+        </r>
+        <r>
+          <t xml:space="preserve">Type: text
+</t>
+        </r>
+        <r>
+          <t xml:space="preserve">CONDITIONAL REPEATABLE — slot #1 of 3 for "Add more drivers?.Driver Information" (Driver).
+Only fill these slots when "Add more drivers?" is set to yes / true.
+Fill slots IN ORDER: slot #1 first, then #2, etc. A gap (e.g. #1 empty but #2 filled) will FAIL the row.
+up to 3 items configured (template provides 3 slots). at least 1 item(s) required when "Add more drivers?" is yes / true.
+Required within filled slot.
+</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AD2" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">Add more drivers?.Driver Information #1 First Name (yes)
+</t>
+        </r>
+        <r>
+          <t xml:space="preserve">Column id: extras.moreDriver__y_c0_r1_firstName
+</t>
+        </r>
+        <r>
+          <t xml:space="preserve">Type: text
+</t>
+        </r>
+        <r>
+          <t xml:space="preserve">CONDITIONAL REPEATABLE — slot #1 of 3 for "Add more drivers?.Driver Information" (Driver).
+Only fill these slots when "Add more drivers?" is set to yes / true.
+Fill slots IN ORDER: slot #1 first, then #2, etc. A gap (e.g. #1 empty but #2 filled) will FAIL the row.
+up to 3 items configured (template provides 3 slots). at least 1 item(s) required when "Add more drivers?" is yes / true.
+</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AF2" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">Add more drivers?.Driver Information #2 Last Name (yes)
+</t>
+        </r>
+        <r>
+          <t xml:space="preserve">Column id: extras.moreDriver__y_c0_r2_lastName
+</t>
+        </r>
+        <r>
+          <t xml:space="preserve">Type: text
+</t>
+        </r>
+        <r>
+          <t xml:space="preserve">CONDITIONAL REPEATABLE — slot #2 of 3 for "Add more drivers?.Driver Information" (Driver).
+Only fill these slots when "Add more drivers?" is set to yes / true.
+Fill slots IN ORDER: slot #1 first, then #2, etc. A gap (e.g. #1 empty but #2 filled) will FAIL the row.
+up to 3 items configured (template provides 3 slots). at least 1 item(s) required when "Add more drivers?" is yes / true.
+Required within filled slot.
+</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AG2" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">Add more drivers?.Driver Information #2 First Name (yes)
+</t>
+        </r>
+        <r>
+          <t xml:space="preserve">Column id: extras.moreDriver__y_c0_r2_firstName
+</t>
+        </r>
+        <r>
+          <t xml:space="preserve">Type: text
+</t>
+        </r>
+        <r>
+          <t xml:space="preserve">CONDITIONAL REPEATABLE — slot #2 of 3 for "Add more drivers?.Driver Information" (Driver).
+Only fill these slots when "Add more drivers?" is set to yes / true.
+Fill slots IN ORDER: slot #1 first, then #2, etc. A gap (e.g. #1 empty but #2 filled) will FAIL the row.
+up to 3 items configured (template provides 3 slots). at least 1 item(s) required when "Add more drivers?" is yes / true.
+</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AI2" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">Add more drivers?.Driver Information #3 Last Name (yes)
+</t>
+        </r>
+        <r>
+          <t xml:space="preserve">Column id: extras.moreDriver__y_c0_r3_lastName
+</t>
+        </r>
+        <r>
+          <t xml:space="preserve">Type: text
+</t>
+        </r>
+        <r>
+          <t xml:space="preserve">CONDITIONAL REPEATABLE — slot #3 of 3 for "Add more drivers?.Driver Information" (Driver).
+Only fill these slots when "Add more drivers?" is set to yes / true.
+Fill slots IN ORDER: slot #1 first, then #2, etc. A gap (e.g. #1 empty but #2 filled) will FAIL the row.
+up to 3 items configured (template provides 3 slots). at least 1 item(s) required when "Add more drivers?" is yes / true.
+Required within filled slot.
+</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AJ2" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">Add more drivers?.Driver Information #3 First Name (yes)
+</t>
+        </r>
+        <r>
+          <t xml:space="preserve">Column id: extras.moreDriver__y_c0_r3_firstName
+</t>
+        </r>
+        <r>
+          <t xml:space="preserve">Type: text
+</t>
+        </r>
+        <r>
+          <t xml:space="preserve">CONDITIONAL REPEATABLE — slot #3 of 3 for "Add more drivers?.Driver Information" (Driver).
+Only fill these slots when "Add more drivers?" is set to yes / true.
+Fill slots IN ORDER: slot #1 first, then #2, etc. A gap (e.g. #1 empty but #2 filled) will FAIL the row.
+up to 3 items configured (template provides 3 slots). at least 1 item(s) required when "Add more drivers?" is yes / true.
+</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="198">
   <si>
     <t>Policy Import Template — Flow: Policy Set (policyset)</t>
   </si>
@@ -427,6 +862,36 @@
     <t xml:space="preserve">  • Filling a column that doesn't apply to the row's type will FAIL the row.</t>
   </si>
   <si>
+    <t>Conditional columns are COLLAPSED by default:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  • To keep the sheet tidy, every column whose meaning depends on another</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    column (boolean children, select option children, etc.) starts hidden</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    inside an Excel column GROUP.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  • Look for the small '+' button just above the column letters bar.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Click '+' to EXPAND a group and reveal its conditional sub-columns.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Click '-' (above the expanded group) to COLLAPSE it again.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  • Cells inside conditional groups also turn pale grey on rows where the</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    parent value doesn't activate them — that's a visual hint that you</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    should NOT type into those cells for that row.</t>
+  </si>
+  <si>
     <t>Boolean conditional fields (tagged '(if yes)' / '(if no)'):</t>
   </si>
   <si>
@@ -457,6 +922,75 @@
     <t xml:space="preserve">  • Only fill them when the parent select equals that option value.</t>
   </si>
   <si>
+    <t>Collapsed select-child fields (tagged '(depends on &lt;parent&gt;)'):</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  • When MANY parent options share the same sub-field shape (e.g. 'Make' has</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    50+ options and each one declares a 'Model' child), we collapse them</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    into ONE column instead of generating 50 redundant 'Model' columns.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  • These columns have no in-cell dropdown because the valid value list</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    changes per parent value. The cell comment lists examples by parent.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  • Make sure your value matches what the wizard would accept for the chosen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    parent value, otherwise the row will FAIL.</t>
+  </si>
+  <si>
+    <t>Repeatable fields (tagged '(item N/M)'):</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  • Lists like 'Drivers' or 'Compensations' get up to 10 numbered slots.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Default is 3 slots when the admin hasn't capped the field.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  • Each slot has its own set of sub-field columns labelled 'Drivers #1 Name',</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    'Drivers #1 Age', 'Drivers #2 Name', 'Drivers #2 Age', etc.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  • Fill slots IN ORDER: slot #1 first, then #2, then #3. Skipping (e.g. #1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    blank but #2 filled) will FAIL the row with a clear error.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  • If the field has a minimum count, the row must fill at least that many slots.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  • Need more slots than the template provides? Re-create the row(s) via the</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    wizard, or split into multiple imports.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  • Boolean-gated repeatable lists (e.g. 'Additional Drivers' shown only when</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    'More Driver?' = yes) get ONE separate '+' button per slot, so you can</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    expand only the driver rows you actually need (driver #2 alone, for</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    instance). A thin blank column between slots is the visual separator —</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    it's intentional and the importer ignores it.</t>
+  </si>
+  <si>
     <t>Client linking:</t>
   </si>
   <si>
@@ -475,7 +1009,13 @@
     <t xml:space="preserve">  • Step 1 — Choosing Insured Type → package "Contact Info" (contactinfo): 2 columns</t>
   </si>
   <si>
-    <t xml:space="preserve">  • Step 2 — Choosing Insurance Type → package "Policy Info" (policyinfo): 9 columns</t>
+    <t xml:space="preserve">  • Step 2 — Choosing Insurance Type → package "Policy Info" (policyinfo): 11 columns</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  • Step 3 — Vehicle Details → package "Vehicle Info" (vehicleinfo): 10 columns</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  • Step 4 — Extras → package "Extras" (extras): 9 columns</t>
   </si>
   <si>
     <t>Field reference (label → column id, type, allowed values / reference):</t>
@@ -526,6 +1066,63 @@
     <t xml:space="preserve">  Policy Info → Type of Cover.Sum Insured (when Comprehensive) → policyinfo.typeOfCover__o_comp_sc0 [currency]  [only when Type of Cover="Comprehensive" (comp)]</t>
   </si>
   <si>
+    <t xml:space="preserve">  Policy Info → Type of Cover.Own Vehicle Damage Cover? (when Third Party Only) → policyinfo.typeOfCover__o_tpo_sc0 [boolean]  [only when Type of Cover="Third Party Only" (tpo)]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Policy Info → Type of Cover.Own Vehicle Damage Cover?.Estimate Value (when Third Party Only / yes) → policyinfo.typeOfCover__o_tpo_sc0__y_bc0 [currency]  [only when Type of Cover="Third Party Only" AND Own Vehicle Damage Cover?=yes]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Vehicle Info → Make → vehicleinfo.make [select] *required  [values: toyota | bmw | honda]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Vehicle Info → Make.Model → vehicleinfo.make__sc0_model [select]  [depends on Make (3 parent options)]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Vehicle Info → Drivers #1 Name → vehicleinfo.drivers__r1_name [text]  [slot 1/4 of "Drivers"; required within filled slot]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Vehicle Info → Drivers #1 Age → vehicleinfo.drivers__r1_age [number]  [slot 1/4 of "Drivers"]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Vehicle Info → Drivers #2 Name → vehicleinfo.drivers__r2_name [text]  [slot 2/4 of "Drivers"; required within filled slot]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Vehicle Info → Drivers #2 Age → vehicleinfo.drivers__r2_age [number]  [slot 2/4 of "Drivers"]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Vehicle Info → Drivers #3 Name → vehicleinfo.drivers__r3_name [text]  [slot 3/4 of "Drivers"; required within filled slot]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Vehicle Info → Drivers #3 Age → vehicleinfo.drivers__r3_age [number]  [slot 3/4 of "Drivers"]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Vehicle Info → Drivers #4 Name → vehicleinfo.drivers__r4_name [text]  [slot 4/4 of "Drivers"; required within filled slot]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Vehicle Info → Drivers #4 Age → vehicleinfo.drivers__r4_age [number]  [slot 4/4 of "Drivers"]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Extras → Add more drivers? → extras.moreDriver [boolean]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Extras → Add more drivers?.Driver Information #1 Last Name (yes) → extras.moreDriver__y_c0_r1_lastName [text]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Extras → Add more drivers?.Driver Information #1 First Name (yes) → extras.moreDriver__y_c0_r1_firstName [text]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Extras → Add more drivers?.Driver Information #2 Last Name (yes) → extras.moreDriver__y_c0_r2_lastName [text]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Extras → Add more drivers?.Driver Information #2 First Name (yes) → extras.moreDriver__y_c0_r2_firstName [text]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Extras → Add more drivers?.Driver Information #3 Last Name (yes) → extras.moreDriver__y_c0_r3_lastName [text]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Extras → Add more drivers?.Driver Information #3 First Name (yes) → extras.moreDriver__y_c0_r3_firstName [text]</t>
+  </si>
+  <si>
     <t>Step 1 — Choosing Insured Type  ›  Insured</t>
   </si>
   <si>
@@ -535,6 +1132,12 @@
     <t>Step 2 — Choosing Insurance Type  ›  Policy Info</t>
   </si>
   <si>
+    <t>Step 3 — Vehicle Details  ›  Vehicle Info</t>
+  </si>
+  <si>
+    <t>Step 4 — Extras  ›  Extras</t>
+  </si>
+  <si>
     <t>Insured Type * (type)</t>
   </si>
   <si>
@@ -580,6 +1183,63 @@
     <t>Type of Cover.Sum Insured (when Comprehensive) (if=comp)</t>
   </si>
   <si>
+    <t>Type of Cover.Own Vehicle Damage Cover? (when Third Party Only) (if=tpo)</t>
+  </si>
+  <si>
+    <t>Type of Cover.Own Vehicle Damage Cover?.Estimate Value (when Third Party Only / yes) (if=tpo/y)</t>
+  </si>
+  <si>
+    <t>Make *</t>
+  </si>
+  <si>
+    <t>Make.Model (depends on Make)</t>
+  </si>
+  <si>
+    <t>Drivers #1 Name (item 1/4)</t>
+  </si>
+  <si>
+    <t>Drivers #1 Age (item 1/4)</t>
+  </si>
+  <si>
+    <t>Drivers #2 Name (item 2/4)</t>
+  </si>
+  <si>
+    <t>Drivers #2 Age (item 2/4)</t>
+  </si>
+  <si>
+    <t>Drivers #3 Name (item 3/4)</t>
+  </si>
+  <si>
+    <t>Drivers #3 Age (item 3/4)</t>
+  </si>
+  <si>
+    <t>Drivers #4 Name (item 4/4)</t>
+  </si>
+  <si>
+    <t>Drivers #4 Age (item 4/4)</t>
+  </si>
+  <si>
+    <t>Add more drivers?</t>
+  </si>
+  <si>
+    <t>Add more drivers?.Driver Information #1 Last Name (yes) (if yes / item 1/3)</t>
+  </si>
+  <si>
+    <t>Add more drivers?.Driver Information #1 First Name (yes) (if yes / item 1/3)</t>
+  </si>
+  <si>
+    <t>Add more drivers?.Driver Information #2 Last Name (yes) (if yes / item 2/3)</t>
+  </si>
+  <si>
+    <t>Add more drivers?.Driver Information #2 First Name (yes) (if yes / item 2/3)</t>
+  </si>
+  <si>
+    <t>Add more drivers?.Driver Information #3 Last Name (yes) (if yes / item 3/3)</t>
+  </si>
+  <si>
+    <t>Add more drivers?.Driver Information #3 First Name (yes) (if yes / item 3/3)</t>
+  </si>
+  <si>
     <t>insured.category</t>
   </si>
   <si>
@@ -625,6 +1285,63 @@
     <t>policyinfo.typeOfCover__o_comp_sc0</t>
   </si>
   <si>
+    <t>policyinfo.typeOfCover__o_tpo_sc0</t>
+  </si>
+  <si>
+    <t>policyinfo.typeOfCover__o_tpo_sc0__y_bc0</t>
+  </si>
+  <si>
+    <t>vehicleinfo.make</t>
+  </si>
+  <si>
+    <t>vehicleinfo.make__sc0_model</t>
+  </si>
+  <si>
+    <t>vehicleinfo.drivers__r1_name</t>
+  </si>
+  <si>
+    <t>vehicleinfo.drivers__r1_age</t>
+  </si>
+  <si>
+    <t>vehicleinfo.drivers__r2_name</t>
+  </si>
+  <si>
+    <t>vehicleinfo.drivers__r2_age</t>
+  </si>
+  <si>
+    <t>vehicleinfo.drivers__r3_name</t>
+  </si>
+  <si>
+    <t>vehicleinfo.drivers__r3_age</t>
+  </si>
+  <si>
+    <t>vehicleinfo.drivers__r4_name</t>
+  </si>
+  <si>
+    <t>vehicleinfo.drivers__r4_age</t>
+  </si>
+  <si>
+    <t>extras.moreDriver</t>
+  </si>
+  <si>
+    <t>extras.moreDriver__y_c0_r1_lastName</t>
+  </si>
+  <si>
+    <t>extras.moreDriver__y_c0_r1_firstName</t>
+  </si>
+  <si>
+    <t>extras.moreDriver__y_c0_r2_lastName</t>
+  </si>
+  <si>
+    <t>extras.moreDriver__y_c0_r2_firstName</t>
+  </si>
+  <si>
+    <t>extras.moreDriver__y_c0_r3_lastName</t>
+  </si>
+  <si>
+    <t>extras.moreDriver__y_c0_r3_firstName</t>
+  </si>
+  <si>
     <t>personal</t>
   </si>
   <si>
@@ -640,10 +1357,13 @@
     <t>31/12/2026</t>
   </si>
   <si>
-    <t>false</t>
+    <t>no</t>
   </si>
   <si>
     <t>tpo</t>
+  </si>
+  <si>
+    <t>toyota</t>
   </si>
 </sst>
 </file>
@@ -681,7 +1401,7 @@
       <color rgb="FFAFAFAF"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -705,6 +1425,16 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFE65100"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFAD1457"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFE8F0FE"/>
       </patternFill>
     </fill>
@@ -714,7 +1444,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -764,11 +1494,33 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="hair">
+        <color rgb="FFE65100"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFB6CCE9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="hair">
+        <color rgb="FFAD1457"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFB6CCE9"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -780,22 +1532,167 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="12">
+    <dxf>
+      <font>
+        <i/>
+        <color rgb="FFB0B0B0"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFF5F5F5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <i/>
+        <color rgb="FFB0B0B0"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFF5F5F5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <i/>
+        <color rgb="FFB0B0B0"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFF5F5F5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <i/>
+        <color rgb="FFB0B0B0"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFF5F5F5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <i/>
+        <color rgb="FFB0B0B0"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFF5F5F5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <i/>
+        <color rgb="FFB0B0B0"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFF5F5F5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <i/>
+        <color rgb="FFB0B0B0"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFF5F5F5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <i/>
+        <color rgb="FFB0B0B0"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFF5F5F5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <i/>
+        <color rgb="FFB0B0B0"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFF5F5F5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <i/>
+        <color rgb="FFB0B0B0"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFF5F5F5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <i/>
+        <color rgb="FFB0B0B0"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFF5F5F5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <i/>
+        <color rgb="FFB0B0B0"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFF5F5F5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -1130,7 +2027,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A71"/>
+  <dimension ref="A1:A128"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="110" customWidth="1"/>
@@ -1328,57 +2225,57 @@
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>1</v>
+        <v>34</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>39</v>
+        <v>1</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>1</v>
+        <v>40</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.25">
@@ -1388,82 +2285,82 @@
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>1</v>
+        <v>48</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>48</v>
+        <v>1</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="63" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="65" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="66" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>57</v>
+        <v>1</v>
       </c>
     </row>
     <row r="67" spans="1:1" x14ac:dyDescent="0.25">
@@ -1489,6 +2386,291 @@
     <row r="71" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>62</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="74" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="75" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="76" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="77" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="78" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="79" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="80" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="81" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="82" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="83" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="84" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="85" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="86" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="87" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="88" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="89" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="90" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="91" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="92" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="93" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="94" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="95" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="96" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="97" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="98" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="99" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="100" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="101" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="102" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="103" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="104" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="105" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="106" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="107" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="108" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="109" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="110" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="111" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="112" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="113" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="114" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="115" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="116" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="117" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="118" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="119" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="120" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="121" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="122" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="123" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="124" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="125" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="126" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A126" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="127" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A127" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="128" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A128" t="s">
+        <v>116</v>
       </c>
     </row>
   </sheetData>
@@ -1499,7 +2681,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O4"/>
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <dimension ref="A1:AJ4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -1512,25 +2697,41 @@
     <col min="9" max="9" width="18" customWidth="1"/>
     <col min="10" max="10" width="19" customWidth="1"/>
     <col min="11" max="11" width="16" customWidth="1"/>
-    <col min="12" max="12" width="32" customWidth="1"/>
-    <col min="13" max="13" width="27" customWidth="1"/>
+    <col min="12" max="12" width="32" hidden="1" outlineLevel="1" collapsed="1" customWidth="1"/>
+    <col min="13" max="13" width="27" hidden="1" outlineLevel="1" collapsed="1" customWidth="1"/>
     <col min="14" max="14" width="19" customWidth="1"/>
-    <col min="15" max="15" width="38" customWidth="1"/>
+    <col min="15" max="17" width="38" hidden="1" outlineLevel="1" collapsed="1" customWidth="1"/>
+    <col min="18" max="18" width="16" customWidth="1"/>
+    <col min="19" max="19" width="16" hidden="1" outlineLevel="1" collapsed="1" customWidth="1"/>
+    <col min="20" max="20" width="21" customWidth="1"/>
+    <col min="21" max="21" width="20" customWidth="1"/>
+    <col min="22" max="22" width="21" customWidth="1"/>
+    <col min="23" max="23" width="20" customWidth="1"/>
+    <col min="24" max="24" width="21" customWidth="1"/>
+    <col min="25" max="25" width="20" customWidth="1"/>
+    <col min="26" max="26" width="21" customWidth="1"/>
+    <col min="27" max="27" width="20" customWidth="1"/>
+    <col min="28" max="28" width="23" customWidth="1"/>
+    <col min="29" max="30" width="38" hidden="1" outlineLevel="1" collapsed="1" customWidth="1"/>
+    <col min="31" max="31" width="2" customWidth="1"/>
+    <col min="32" max="33" width="38" hidden="1" outlineLevel="1" collapsed="1" customWidth="1"/>
+    <col min="34" max="34" width="2" customWidth="1"/>
+    <col min="35" max="36" width="38" hidden="1" outlineLevel="1" collapsed="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" ht="26" customHeight="1" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>63</v>
+        <v>117</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
       <c r="E1" s="3" t="s">
-        <v>64</v>
+        <v>118</v>
       </c>
       <c r="F1" s="3"/>
       <c r="G1" s="4" t="s">
-        <v>65</v>
+        <v>119</v>
       </c>
       <c r="H1" s="4"/>
       <c r="I1" s="4"/>
@@ -1540,167 +2741,434 @@
       <c r="M1" s="4"/>
       <c r="N1" s="4"/>
       <c r="O1" s="4"/>
-    </row>
-    <row r="2" ht="30" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>68</v>
-      </c>
-      <c r="D2" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="E2" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="F2" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="G2" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="H2" s="7" t="s">
-        <v>73</v>
-      </c>
-      <c r="I2" s="7" t="s">
-        <v>74</v>
-      </c>
-      <c r="J2" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="K2" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="L2" s="7" t="s">
-        <v>77</v>
-      </c>
-      <c r="M2" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="N2" s="7" t="s">
-        <v>79</v>
-      </c>
-      <c r="O2" s="7" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="3" ht="14" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A3" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="B3" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="C3" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="D3" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="E3" s="8" t="s">
-        <v>85</v>
-      </c>
-      <c r="F3" s="8" t="s">
-        <v>86</v>
-      </c>
-      <c r="G3" s="8" t="s">
-        <v>87</v>
-      </c>
-      <c r="H3" s="8" t="s">
-        <v>88</v>
-      </c>
-      <c r="I3" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="J3" s="8" t="s">
-        <v>90</v>
-      </c>
-      <c r="K3" s="8" t="s">
-        <v>91</v>
-      </c>
-      <c r="L3" s="8" t="s">
-        <v>92</v>
-      </c>
-      <c r="M3" s="8" t="s">
-        <v>93</v>
-      </c>
-      <c r="N3" s="8" t="s">
-        <v>94</v>
-      </c>
-      <c r="O3" s="8" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A4" s="9" t="s">
-        <v>96</v>
-      </c>
-      <c r="B4" s="9" t="s">
-        <v>1</v>
-      </c>
-      <c r="C4" s="9" t="s">
-        <v>1</v>
-      </c>
-      <c r="D4" s="9" t="s">
-        <v>97</v>
-      </c>
-      <c r="E4" s="9" t="s">
-        <v>98</v>
-      </c>
-      <c r="F4" s="9" t="s">
-        <v>99</v>
-      </c>
-      <c r="G4" s="9" t="s">
-        <v>1</v>
-      </c>
-      <c r="H4" s="9" t="s">
-        <v>1</v>
-      </c>
-      <c r="I4" s="9" t="s">
-        <v>100</v>
-      </c>
-      <c r="J4" s="9" t="s">
-        <v>99</v>
-      </c>
-      <c r="K4" s="9" t="s">
-        <v>101</v>
-      </c>
-      <c r="L4" s="9" t="s">
-        <v>1</v>
-      </c>
-      <c r="M4" s="9" t="s">
-        <v>1</v>
-      </c>
-      <c r="N4" s="9" t="s">
-        <v>102</v>
-      </c>
-      <c r="O4" s="9" t="s">
+      <c r="P1" s="4"/>
+      <c r="Q1" s="4"/>
+      <c r="R1" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="S1" s="5"/>
+      <c r="T1" s="5"/>
+      <c r="U1" s="5"/>
+      <c r="V1" s="5"/>
+      <c r="W1" s="5"/>
+      <c r="X1" s="5"/>
+      <c r="Y1" s="5"/>
+      <c r="Z1" s="5"/>
+      <c r="AA1" s="5"/>
+      <c r="AB1" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="AC1" s="6"/>
+      <c r="AD1" s="6"/>
+      <c r="AE1" s="6"/>
+      <c r="AF1" s="6"/>
+      <c r="AG1" s="6"/>
+      <c r="AH1" s="6"/>
+      <c r="AI1" s="6"/>
+      <c r="AJ1" s="6"/>
+    </row>
+    <row r="2" ht="30" customHeight="1" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A2" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="E2" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="G2" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="H2" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="I2" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="J2" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="K2" s="9" t="s">
+        <v>132</v>
+      </c>
+      <c r="L2" s="9" t="s">
+        <v>133</v>
+      </c>
+      <c r="M2" s="9" t="s">
+        <v>134</v>
+      </c>
+      <c r="N2" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="O2" s="9" t="s">
+        <v>136</v>
+      </c>
+      <c r="P2" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="Q2" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="R2" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="S2" s="10" t="s">
+        <v>140</v>
+      </c>
+      <c r="T2" s="10" t="s">
+        <v>141</v>
+      </c>
+      <c r="U2" s="10" t="s">
+        <v>142</v>
+      </c>
+      <c r="V2" s="10" t="s">
+        <v>143</v>
+      </c>
+      <c r="W2" s="10" t="s">
+        <v>144</v>
+      </c>
+      <c r="X2" s="10" t="s">
+        <v>145</v>
+      </c>
+      <c r="Y2" s="10" t="s">
+        <v>146</v>
+      </c>
+      <c r="Z2" s="10" t="s">
+        <v>147</v>
+      </c>
+      <c r="AA2" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="AB2" s="11" t="s">
+        <v>149</v>
+      </c>
+      <c r="AC2" s="11" t="s">
+        <v>150</v>
+      </c>
+      <c r="AD2" s="11" t="s">
+        <v>151</v>
+      </c>
+      <c r="AF2" s="11" t="s">
+        <v>152</v>
+      </c>
+      <c r="AG2" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="AI2" s="11" t="s">
+        <v>154</v>
+      </c>
+      <c r="AJ2" s="11" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="3" ht="14" customHeight="1" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A3" s="12" t="s">
+        <v>156</v>
+      </c>
+      <c r="B3" s="12" t="s">
+        <v>157</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>158</v>
+      </c>
+      <c r="D3" s="12" t="s">
+        <v>159</v>
+      </c>
+      <c r="E3" s="12" t="s">
+        <v>160</v>
+      </c>
+      <c r="F3" s="12" t="s">
+        <v>161</v>
+      </c>
+      <c r="G3" s="12" t="s">
+        <v>162</v>
+      </c>
+      <c r="H3" s="12" t="s">
+        <v>163</v>
+      </c>
+      <c r="I3" s="12" t="s">
+        <v>164</v>
+      </c>
+      <c r="J3" s="12" t="s">
+        <v>165</v>
+      </c>
+      <c r="K3" s="12" t="s">
+        <v>166</v>
+      </c>
+      <c r="L3" s="12" t="s">
+        <v>167</v>
+      </c>
+      <c r="M3" s="12" t="s">
+        <v>168</v>
+      </c>
+      <c r="N3" s="12" t="s">
+        <v>169</v>
+      </c>
+      <c r="O3" s="12" t="s">
+        <v>170</v>
+      </c>
+      <c r="P3" s="12" t="s">
+        <v>171</v>
+      </c>
+      <c r="Q3" s="12" t="s">
+        <v>172</v>
+      </c>
+      <c r="R3" s="12" t="s">
+        <v>173</v>
+      </c>
+      <c r="S3" s="12" t="s">
+        <v>174</v>
+      </c>
+      <c r="T3" s="12" t="s">
+        <v>175</v>
+      </c>
+      <c r="U3" s="12" t="s">
+        <v>176</v>
+      </c>
+      <c r="V3" s="12" t="s">
+        <v>177</v>
+      </c>
+      <c r="W3" s="12" t="s">
+        <v>178</v>
+      </c>
+      <c r="X3" s="12" t="s">
+        <v>179</v>
+      </c>
+      <c r="Y3" s="12" t="s">
+        <v>180</v>
+      </c>
+      <c r="Z3" s="12" t="s">
+        <v>181</v>
+      </c>
+      <c r="AA3" s="12" t="s">
+        <v>182</v>
+      </c>
+      <c r="AB3" s="12" t="s">
+        <v>183</v>
+      </c>
+      <c r="AC3" s="12" t="s">
+        <v>184</v>
+      </c>
+      <c r="AD3" s="12" t="s">
+        <v>185</v>
+      </c>
+      <c r="AF3" s="12" t="s">
+        <v>186</v>
+      </c>
+      <c r="AG3" s="12" t="s">
+        <v>187</v>
+      </c>
+      <c r="AI3" s="12" t="s">
+        <v>188</v>
+      </c>
+      <c r="AJ3" s="12" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A4" s="13" t="s">
+        <v>190</v>
+      </c>
+      <c r="B4" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="D4" s="13" t="s">
+        <v>191</v>
+      </c>
+      <c r="E4" s="13" t="s">
+        <v>192</v>
+      </c>
+      <c r="F4" s="13" t="s">
+        <v>193</v>
+      </c>
+      <c r="G4" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="H4" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="I4" s="13" t="s">
+        <v>194</v>
+      </c>
+      <c r="J4" s="13" t="s">
+        <v>193</v>
+      </c>
+      <c r="K4" s="13" t="s">
+        <v>195</v>
+      </c>
+      <c r="L4" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="M4" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="N4" s="13" t="s">
+        <v>196</v>
+      </c>
+      <c r="O4" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="P4" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="Q4" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="R4" s="13" t="s">
+        <v>197</v>
+      </c>
+      <c r="S4" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="T4" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="U4" s="13" t="s">
+        <v>193</v>
+      </c>
+      <c r="V4" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="W4" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="X4" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="Y4" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="Z4" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="AA4" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="AB4" s="13" t="s">
+        <v>195</v>
+      </c>
+      <c r="AC4" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="AD4" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="AF4" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="AG4" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="AI4" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="AJ4" s="13" t="s">
         <v>1</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:O2"/>
-  <mergeCells count="3">
+  <autoFilter ref="A2:AJ2"/>
+  <mergeCells count="5">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="E1:F1"/>
-    <mergeCell ref="G1:O1"/>
+    <mergeCell ref="G1:Q1"/>
+    <mergeCell ref="R1:AA1"/>
+    <mergeCell ref="AB1:AJ1"/>
   </mergeCells>
-  <dataValidations count="4">
+  <conditionalFormatting sqref="L5:L504">
+    <cfRule type="expression" dxfId="0" priority="1">
+      <formula>AND($K5&lt;&gt;"yes",$K5&lt;&gt;"y",$K5&lt;&gt;"true",$K5&lt;&gt;"1")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M5:M504">
+    <cfRule type="expression" dxfId="1" priority="1">
+      <formula>AND($K5&lt;&gt;"no",$K5&lt;&gt;"n",$K5&lt;&gt;"false",$K5&lt;&gt;"0")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O5:O504">
+    <cfRule type="expression" dxfId="2" priority="1">
+      <formula>$N5&lt;&gt;"comp"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="P5:P504">
+    <cfRule type="expression" dxfId="3" priority="1">
+      <formula>$N5&lt;&gt;"tpo"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q5:Q504">
+    <cfRule type="expression" dxfId="4" priority="1">
+      <formula>OR($N5&lt;&gt;"tpo",AND($P5&lt;&gt;"yes",$P5&lt;&gt;"y",$P5&lt;&gt;"true",$P5&lt;&gt;"1"))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S5:S504">
+    <cfRule type="expression" dxfId="5" priority="1">
+      <formula>AND($R5&lt;&gt;"toyota",$R5&lt;&gt;"bmw",$R5&lt;&gt;"honda")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AC5:AC504">
+    <cfRule type="expression" dxfId="6" priority="1">
+      <formula>AND($AB5&lt;&gt;"yes",$AB5&lt;&gt;"y",$AB5&lt;&gt;"true",$AB5&lt;&gt;"1")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AD5:AD504">
+    <cfRule type="expression" dxfId="7" priority="1">
+      <formula>AND($AB5&lt;&gt;"yes",$AB5&lt;&gt;"y",$AB5&lt;&gt;"true",$AB5&lt;&gt;"1")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AF5:AF504">
+    <cfRule type="expression" dxfId="8" priority="1">
+      <formula>AND($AB5&lt;&gt;"yes",$AB5&lt;&gt;"y",$AB5&lt;&gt;"true",$AB5&lt;&gt;"1")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AG5:AG504">
+    <cfRule type="expression" dxfId="9" priority="1">
+      <formula>AND($AB5&lt;&gt;"yes",$AB5&lt;&gt;"y",$AB5&lt;&gt;"true",$AB5&lt;&gt;"1")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AI5:AI504">
+    <cfRule type="expression" dxfId="10" priority="1">
+      <formula>AND($AB5&lt;&gt;"yes",$AB5&lt;&gt;"y",$AB5&lt;&gt;"true",$AB5&lt;&gt;"1")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AJ5:AJ504">
+    <cfRule type="expression" dxfId="11" priority="1">
+      <formula>AND($AB5&lt;&gt;"yes",$AB5&lt;&gt;"y",$AB5&lt;&gt;"true",$AB5&lt;&gt;"1")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="7">
     <dataValidation type="list" showErrorMessage="1" errorStyle="warning" errorTitle="Invalid value" error="Allowed: personal, company" sqref="A4:A504">
       <formula1>"personal,company"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" sqref="AB4:AB504">
+      <formula1>"yes,no"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="Invalid value" error="Allowed: hk, hkc, qc" sqref="D4:D504">
       <formula1>"hk,hkc,qc"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" sqref="K4:K504">
-      <formula1>"true,false,yes,no"</formula1>
+      <formula1>"yes,no"</formula1>
     </dataValidation>
     <dataValidation type="list" showErrorMessage="1" errorStyle="warning" errorTitle="Invalid value" error="Allowed: tpo, comp" sqref="N4:N504">
       <formula1>"tpo,comp"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" sqref="P4:P504">
+      <formula1>"yes,no"</formula1>
+    </dataValidation>
+    <dataValidation type="list" showErrorMessage="1" errorStyle="warning" errorTitle="Invalid value" error="Allowed: toyota, bmw, honda" sqref="R4:R504">
+      <formula1>"toyota,bmw,honda"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
import excel form 2
</commit_message>
<xml_diff>
--- a/scripts/_smoke-template.xlsx
+++ b/scripts/_smoke-template.xlsx
@@ -671,7 +671,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AF2" authorId="0">
+    <comment ref="AE2" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Add more drivers?.Driver Information #2 Last Name (yes)
@@ -695,7 +695,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AG2" authorId="0">
+    <comment ref="AF2" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Add more drivers?.Driver Information #2 First Name (yes)
@@ -718,7 +718,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AI2" authorId="0">
+    <comment ref="AG2" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Add more drivers?.Driver Information #3 Last Name (yes)
@@ -742,7 +742,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AJ2" authorId="0">
+    <comment ref="AH2" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Add more drivers?.Driver Information #3 First Name (yes)
@@ -770,7 +770,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="198">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="183">
   <si>
     <t>Policy Import Template — Flow: Policy Set (policyset)</t>
   </si>
@@ -862,36 +862,6 @@
     <t xml:space="preserve">  • Filling a column that doesn't apply to the row's type will FAIL the row.</t>
   </si>
   <si>
-    <t>Conditional columns are COLLAPSED by default:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  • To keep the sheet tidy, every column whose meaning depends on another</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    column (boolean children, select option children, etc.) starts hidden</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    inside an Excel column GROUP.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  • Look for the small '+' button just above the column letters bar.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    Click '+' to EXPAND a group and reveal its conditional sub-columns.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    Click '-' (above the expanded group) to COLLAPSE it again.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  • Cells inside conditional groups also turn pale grey on rows where the</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    parent value doesn't activate them — that's a visual hint that you</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    should NOT type into those cells for that row.</t>
-  </si>
-  <si>
     <t>Boolean conditional fields (tagged '(if yes)' / '(if no)'):</t>
   </si>
   <si>
@@ -976,21 +946,6 @@
     <t xml:space="preserve">    wizard, or split into multiple imports.</t>
   </si>
   <si>
-    <t xml:space="preserve">  • Boolean-gated repeatable lists (e.g. 'Additional Drivers' shown only when</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    'More Driver?' = yes) get ONE separate '+' button per slot, so you can</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    expand only the driver rows you actually need (driver #2 alone, for</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    instance). A thin blank column between slots is the visual separator —</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    it's intentional and the importer ignores it.</t>
-  </si>
-  <si>
     <t>Client linking:</t>
   </si>
   <si>
@@ -1015,7 +970,7 @@
     <t xml:space="preserve">  • Step 3 — Vehicle Details → package "Vehicle Info" (vehicleinfo): 10 columns</t>
   </si>
   <si>
-    <t xml:space="preserve">  • Step 4 — Extras → package "Extras" (extras): 9 columns</t>
+    <t xml:space="preserve">  • Step 4 — Extras → package "Extras" (extras): 7 columns</t>
   </si>
   <si>
     <t>Field reference (label → column id, type, allowed values / reference):</t>
@@ -1138,7 +1093,7 @@
     <t>Step 4 — Extras  ›  Extras</t>
   </si>
   <si>
-    <t>Insured Type * (type)</t>
+    <t>Insured Type * (type) [personal|company]</t>
   </si>
   <si>
     <t>First Name * [personal]</t>
@@ -1559,140 +1514,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="12">
-    <dxf>
-      <font>
-        <i/>
-        <color rgb="FFB0B0B0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFF5F5F5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <i/>
-        <color rgb="FFB0B0B0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFF5F5F5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <i/>
-        <color rgb="FFB0B0B0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFF5F5F5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <i/>
-        <color rgb="FFB0B0B0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFF5F5F5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <i/>
-        <color rgb="FFB0B0B0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFF5F5F5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <i/>
-        <color rgb="FFB0B0B0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFF5F5F5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <i/>
-        <color rgb="FFB0B0B0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFF5F5F5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <i/>
-        <color rgb="FFB0B0B0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFF5F5F5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <i/>
-        <color rgb="FFB0B0B0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFF5F5F5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <i/>
-        <color rgb="FFB0B0B0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFF5F5F5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <i/>
-        <color rgb="FFB0B0B0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFF5F5F5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <i/>
-        <color rgb="FFB0B0B0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFF5F5F5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -2027,7 +1849,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A128"/>
+  <dimension ref="A1:A112"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="110" customWidth="1"/>
@@ -2225,62 +2047,62 @@
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>34</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>1</v>
+        <v>39</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>40</v>
+        <v>1</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>1</v>
+        <v>43</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.25">
@@ -2305,17 +2127,17 @@
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>48</v>
+        <v>1</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>1</v>
+        <v>49</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.25">
@@ -2380,87 +2202,87 @@
     </row>
     <row r="70" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>61</v>
+        <v>1</v>
       </c>
     </row>
     <row r="71" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="72" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="73" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="74" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="75" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="76" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="77" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>68</v>
+        <v>1</v>
       </c>
     </row>
     <row r="78" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="79" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="80" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="81" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="82" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>1</v>
+        <v>71</v>
       </c>
     </row>
     <row r="83" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="84" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="85" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="86" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>1</v>
+        <v>75</v>
       </c>
     </row>
     <row r="87" spans="1:1" x14ac:dyDescent="0.25">
@@ -2495,182 +2317,102 @@
     </row>
     <row r="93" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>1</v>
+        <v>82</v>
       </c>
     </row>
     <row r="94" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="95" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="96" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="97" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="98" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="99" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="100" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="101" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="102" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="103" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="104" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="105" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="106" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="107" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="108" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="109" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="110" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="111" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="112" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="113" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A113" t="s">
         <v>101</v>
-      </c>
-    </row>
-    <row r="114" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A114" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="115" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A115" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="116" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A116" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="117" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A117" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="118" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A118" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="119" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A119" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="120" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A120" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="121" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A121" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="122" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A122" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="123" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A123" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="124" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A124" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="125" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A125" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="126" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A126" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="127" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A127" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="128" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A128" t="s">
-        <v>116</v>
       </c>
     </row>
   </sheetData>
@@ -2681,10 +2423,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-  </sheetPr>
-  <dimension ref="A1:AJ4"/>
+  <dimension ref="A1:AH4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -2697,12 +2436,11 @@
     <col min="9" max="9" width="18" customWidth="1"/>
     <col min="10" max="10" width="19" customWidth="1"/>
     <col min="11" max="11" width="16" customWidth="1"/>
-    <col min="12" max="12" width="32" hidden="1" outlineLevel="1" collapsed="1" customWidth="1"/>
-    <col min="13" max="13" width="27" hidden="1" outlineLevel="1" collapsed="1" customWidth="1"/>
+    <col min="12" max="12" width="32" customWidth="1"/>
+    <col min="13" max="13" width="27" customWidth="1"/>
     <col min="14" max="14" width="19" customWidth="1"/>
-    <col min="15" max="17" width="38" hidden="1" outlineLevel="1" collapsed="1" customWidth="1"/>
-    <col min="18" max="18" width="16" customWidth="1"/>
-    <col min="19" max="19" width="16" hidden="1" outlineLevel="1" collapsed="1" customWidth="1"/>
+    <col min="15" max="17" width="38" customWidth="1"/>
+    <col min="18" max="19" width="16" customWidth="1"/>
     <col min="20" max="20" width="21" customWidth="1"/>
     <col min="21" max="21" width="20" customWidth="1"/>
     <col min="22" max="22" width="21" customWidth="1"/>
@@ -2712,26 +2450,22 @@
     <col min="26" max="26" width="21" customWidth="1"/>
     <col min="27" max="27" width="20" customWidth="1"/>
     <col min="28" max="28" width="23" customWidth="1"/>
-    <col min="29" max="30" width="38" hidden="1" outlineLevel="1" collapsed="1" customWidth="1"/>
-    <col min="31" max="31" width="2" customWidth="1"/>
-    <col min="32" max="33" width="38" hidden="1" outlineLevel="1" collapsed="1" customWidth="1"/>
-    <col min="34" max="34" width="2" customWidth="1"/>
-    <col min="35" max="36" width="38" hidden="1" outlineLevel="1" collapsed="1" customWidth="1"/>
+    <col min="29" max="34" width="38" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" ht="26" customHeight="1" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>117</v>
+        <v>102</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
       <c r="E1" s="3" t="s">
-        <v>118</v>
+        <v>103</v>
       </c>
       <c r="F1" s="3"/>
       <c r="G1" s="4" t="s">
-        <v>119</v>
+        <v>104</v>
       </c>
       <c r="H1" s="4"/>
       <c r="I1" s="4"/>
@@ -2744,7 +2478,7 @@
       <c r="P1" s="4"/>
       <c r="Q1" s="4"/>
       <c r="R1" s="5" t="s">
-        <v>120</v>
+        <v>105</v>
       </c>
       <c r="S1" s="5"/>
       <c r="T1" s="5"/>
@@ -2756,7 +2490,7 @@
       <c r="Z1" s="5"/>
       <c r="AA1" s="5"/>
       <c r="AB1" s="6" t="s">
-        <v>121</v>
+        <v>106</v>
       </c>
       <c r="AC1" s="6"/>
       <c r="AD1" s="6"/>
@@ -2764,272 +2498,270 @@
       <c r="AF1" s="6"/>
       <c r="AG1" s="6"/>
       <c r="AH1" s="6"/>
-      <c r="AI1" s="6"/>
-      <c r="AJ1" s="6"/>
-    </row>
-    <row r="2" ht="30" customHeight="1" spans="1:36" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" ht="30" customHeight="1" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="E2" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="G2" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="H2" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="I2" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="J2" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="K2" s="9" t="s">
+        <v>117</v>
+      </c>
+      <c r="L2" s="9" t="s">
+        <v>118</v>
+      </c>
+      <c r="M2" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="N2" s="9" t="s">
+        <v>120</v>
+      </c>
+      <c r="O2" s="9" t="s">
+        <v>121</v>
+      </c>
+      <c r="P2" s="9" t="s">
         <v>122</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="Q2" s="9" t="s">
         <v>123</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="R2" s="10" t="s">
         <v>124</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="S2" s="10" t="s">
         <v>125</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="T2" s="10" t="s">
         <v>126</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="U2" s="10" t="s">
         <v>127</v>
       </c>
-      <c r="G2" s="9" t="s">
+      <c r="V2" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="H2" s="9" t="s">
+      <c r="W2" s="10" t="s">
         <v>129</v>
       </c>
-      <c r="I2" s="9" t="s">
+      <c r="X2" s="10" t="s">
         <v>130</v>
       </c>
-      <c r="J2" s="9" t="s">
+      <c r="Y2" s="10" t="s">
         <v>131</v>
       </c>
-      <c r="K2" s="9" t="s">
+      <c r="Z2" s="10" t="s">
         <v>132</v>
       </c>
-      <c r="L2" s="9" t="s">
+      <c r="AA2" s="10" t="s">
         <v>133</v>
       </c>
-      <c r="M2" s="9" t="s">
+      <c r="AB2" s="11" t="s">
         <v>134</v>
       </c>
-      <c r="N2" s="9" t="s">
+      <c r="AC2" s="11" t="s">
         <v>135</v>
       </c>
-      <c r="O2" s="9" t="s">
+      <c r="AD2" s="11" t="s">
         <v>136</v>
       </c>
-      <c r="P2" s="9" t="s">
+      <c r="AE2" s="11" t="s">
         <v>137</v>
       </c>
-      <c r="Q2" s="9" t="s">
+      <c r="AF2" s="11" t="s">
         <v>138</v>
       </c>
-      <c r="R2" s="10" t="s">
+      <c r="AG2" s="11" t="s">
         <v>139</v>
       </c>
-      <c r="S2" s="10" t="s">
+      <c r="AH2" s="11" t="s">
         <v>140</v>
       </c>
-      <c r="T2" s="10" t="s">
+    </row>
+    <row r="3" ht="14" customHeight="1" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A3" s="12" t="s">
         <v>141</v>
       </c>
-      <c r="U2" s="10" t="s">
+      <c r="B3" s="12" t="s">
         <v>142</v>
       </c>
-      <c r="V2" s="10" t="s">
+      <c r="C3" s="12" t="s">
         <v>143</v>
       </c>
-      <c r="W2" s="10" t="s">
+      <c r="D3" s="12" t="s">
         <v>144</v>
       </c>
-      <c r="X2" s="10" t="s">
+      <c r="E3" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="Y2" s="10" t="s">
+      <c r="F3" s="12" t="s">
         <v>146</v>
       </c>
-      <c r="Z2" s="10" t="s">
+      <c r="G3" s="12" t="s">
         <v>147</v>
       </c>
-      <c r="AA2" s="10" t="s">
+      <c r="H3" s="12" t="s">
         <v>148</v>
       </c>
-      <c r="AB2" s="11" t="s">
+      <c r="I3" s="12" t="s">
         <v>149</v>
       </c>
-      <c r="AC2" s="11" t="s">
+      <c r="J3" s="12" t="s">
         <v>150</v>
       </c>
-      <c r="AD2" s="11" t="s">
+      <c r="K3" s="12" t="s">
         <v>151</v>
       </c>
-      <c r="AF2" s="11" t="s">
+      <c r="L3" s="12" t="s">
         <v>152</v>
       </c>
-      <c r="AG2" s="11" t="s">
+      <c r="M3" s="12" t="s">
         <v>153</v>
       </c>
-      <c r="AI2" s="11" t="s">
+      <c r="N3" s="12" t="s">
         <v>154</v>
       </c>
-      <c r="AJ2" s="11" t="s">
+      <c r="O3" s="12" t="s">
         <v>155</v>
       </c>
-    </row>
-    <row r="3" ht="14" customHeight="1" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A3" s="12" t="s">
+      <c r="P3" s="12" t="s">
         <v>156</v>
       </c>
-      <c r="B3" s="12" t="s">
+      <c r="Q3" s="12" t="s">
         <v>157</v>
       </c>
-      <c r="C3" s="12" t="s">
+      <c r="R3" s="12" t="s">
         <v>158</v>
       </c>
-      <c r="D3" s="12" t="s">
+      <c r="S3" s="12" t="s">
         <v>159</v>
       </c>
-      <c r="E3" s="12" t="s">
+      <c r="T3" s="12" t="s">
         <v>160</v>
       </c>
-      <c r="F3" s="12" t="s">
+      <c r="U3" s="12" t="s">
         <v>161</v>
       </c>
-      <c r="G3" s="12" t="s">
+      <c r="V3" s="12" t="s">
         <v>162</v>
       </c>
-      <c r="H3" s="12" t="s">
+      <c r="W3" s="12" t="s">
         <v>163</v>
       </c>
-      <c r="I3" s="12" t="s">
+      <c r="X3" s="12" t="s">
         <v>164</v>
       </c>
-      <c r="J3" s="12" t="s">
+      <c r="Y3" s="12" t="s">
         <v>165</v>
       </c>
-      <c r="K3" s="12" t="s">
+      <c r="Z3" s="12" t="s">
         <v>166</v>
       </c>
-      <c r="L3" s="12" t="s">
+      <c r="AA3" s="12" t="s">
         <v>167</v>
       </c>
-      <c r="M3" s="12" t="s">
+      <c r="AB3" s="12" t="s">
         <v>168</v>
       </c>
-      <c r="N3" s="12" t="s">
+      <c r="AC3" s="12" t="s">
         <v>169</v>
       </c>
-      <c r="O3" s="12" t="s">
+      <c r="AD3" s="12" t="s">
         <v>170</v>
       </c>
-      <c r="P3" s="12" t="s">
+      <c r="AE3" s="12" t="s">
         <v>171</v>
       </c>
-      <c r="Q3" s="12" t="s">
+      <c r="AF3" s="12" t="s">
         <v>172</v>
       </c>
-      <c r="R3" s="12" t="s">
+      <c r="AG3" s="12" t="s">
         <v>173</v>
       </c>
-      <c r="S3" s="12" t="s">
+      <c r="AH3" s="12" t="s">
         <v>174</v>
       </c>
-      <c r="T3" s="12" t="s">
+    </row>
+    <row r="4" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A4" s="13" t="s">
         <v>175</v>
       </c>
-      <c r="U3" s="12" t="s">
+      <c r="B4" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="D4" s="13" t="s">
         <v>176</v>
       </c>
-      <c r="V3" s="12" t="s">
+      <c r="E4" s="13" t="s">
         <v>177</v>
       </c>
-      <c r="W3" s="12" t="s">
+      <c r="F4" s="13" t="s">
         <v>178</v>
       </c>
-      <c r="X3" s="12" t="s">
+      <c r="G4" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="H4" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="I4" s="13" t="s">
         <v>179</v>
       </c>
-      <c r="Y3" s="12" t="s">
+      <c r="J4" s="13" t="s">
+        <v>178</v>
+      </c>
+      <c r="K4" s="13" t="s">
         <v>180</v>
       </c>
-      <c r="Z3" s="12" t="s">
+      <c r="L4" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="M4" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="N4" s="13" t="s">
         <v>181</v>
       </c>
-      <c r="AA3" s="12" t="s">
+      <c r="O4" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="P4" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="Q4" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="R4" s="13" t="s">
         <v>182</v>
       </c>
-      <c r="AB3" s="12" t="s">
-        <v>183</v>
-      </c>
-      <c r="AC3" s="12" t="s">
-        <v>184</v>
-      </c>
-      <c r="AD3" s="12" t="s">
-        <v>185</v>
-      </c>
-      <c r="AF3" s="12" t="s">
-        <v>186</v>
-      </c>
-      <c r="AG3" s="12" t="s">
-        <v>187</v>
-      </c>
-      <c r="AI3" s="12" t="s">
-        <v>188</v>
-      </c>
-      <c r="AJ3" s="12" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A4" s="13" t="s">
-        <v>190</v>
-      </c>
-      <c r="B4" s="13" t="s">
-        <v>1</v>
-      </c>
-      <c r="C4" s="13" t="s">
-        <v>1</v>
-      </c>
-      <c r="D4" s="13" t="s">
-        <v>191</v>
-      </c>
-      <c r="E4" s="13" t="s">
-        <v>192</v>
-      </c>
-      <c r="F4" s="13" t="s">
-        <v>193</v>
-      </c>
-      <c r="G4" s="13" t="s">
-        <v>1</v>
-      </c>
-      <c r="H4" s="13" t="s">
-        <v>1</v>
-      </c>
-      <c r="I4" s="13" t="s">
-        <v>194</v>
-      </c>
-      <c r="J4" s="13" t="s">
-        <v>193</v>
-      </c>
-      <c r="K4" s="13" t="s">
-        <v>195</v>
-      </c>
-      <c r="L4" s="13" t="s">
-        <v>1</v>
-      </c>
-      <c r="M4" s="13" t="s">
-        <v>1</v>
-      </c>
-      <c r="N4" s="13" t="s">
-        <v>196</v>
-      </c>
-      <c r="O4" s="13" t="s">
-        <v>1</v>
-      </c>
-      <c r="P4" s="13" t="s">
-        <v>1</v>
-      </c>
-      <c r="Q4" s="13" t="s">
-        <v>1</v>
-      </c>
-      <c r="R4" s="13" t="s">
-        <v>197</v>
-      </c>
       <c r="S4" s="13" t="s">
         <v>1</v>
       </c>
@@ -3037,7 +2769,7 @@
         <v>1</v>
       </c>
       <c r="U4" s="13" t="s">
-        <v>193</v>
+        <v>178</v>
       </c>
       <c r="V4" s="13" t="s">
         <v>1</v>
@@ -3058,7 +2790,7 @@
         <v>1</v>
       </c>
       <c r="AB4" s="13" t="s">
-        <v>195</v>
+        <v>180</v>
       </c>
       <c r="AC4" s="13" t="s">
         <v>1</v>
@@ -3066,88 +2798,28 @@
       <c r="AD4" s="13" t="s">
         <v>1</v>
       </c>
+      <c r="AE4" s="13" t="s">
+        <v>1</v>
+      </c>
       <c r="AF4" s="13" t="s">
         <v>1</v>
       </c>
       <c r="AG4" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="AI4" s="13" t="s">
-        <v>1</v>
-      </c>
-      <c r="AJ4" s="13" t="s">
+      <c r="AH4" s="13" t="s">
         <v>1</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:AJ2"/>
+  <autoFilter ref="A2:AH2"/>
   <mergeCells count="5">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="E1:F1"/>
     <mergeCell ref="G1:Q1"/>
     <mergeCell ref="R1:AA1"/>
-    <mergeCell ref="AB1:AJ1"/>
+    <mergeCell ref="AB1:AH1"/>
   </mergeCells>
-  <conditionalFormatting sqref="L5:L504">
-    <cfRule type="expression" dxfId="0" priority="1">
-      <formula>AND($K5&lt;&gt;"yes",$K5&lt;&gt;"y",$K5&lt;&gt;"true",$K5&lt;&gt;"1")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="M5:M504">
-    <cfRule type="expression" dxfId="1" priority="1">
-      <formula>AND($K5&lt;&gt;"no",$K5&lt;&gt;"n",$K5&lt;&gt;"false",$K5&lt;&gt;"0")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="O5:O504">
-    <cfRule type="expression" dxfId="2" priority="1">
-      <formula>$N5&lt;&gt;"comp"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="P5:P504">
-    <cfRule type="expression" dxfId="3" priority="1">
-      <formula>$N5&lt;&gt;"tpo"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q5:Q504">
-    <cfRule type="expression" dxfId="4" priority="1">
-      <formula>OR($N5&lt;&gt;"tpo",AND($P5&lt;&gt;"yes",$P5&lt;&gt;"y",$P5&lt;&gt;"true",$P5&lt;&gt;"1"))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="S5:S504">
-    <cfRule type="expression" dxfId="5" priority="1">
-      <formula>AND($R5&lt;&gt;"toyota",$R5&lt;&gt;"bmw",$R5&lt;&gt;"honda")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AC5:AC504">
-    <cfRule type="expression" dxfId="6" priority="1">
-      <formula>AND($AB5&lt;&gt;"yes",$AB5&lt;&gt;"y",$AB5&lt;&gt;"true",$AB5&lt;&gt;"1")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AD5:AD504">
-    <cfRule type="expression" dxfId="7" priority="1">
-      <formula>AND($AB5&lt;&gt;"yes",$AB5&lt;&gt;"y",$AB5&lt;&gt;"true",$AB5&lt;&gt;"1")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AF5:AF504">
-    <cfRule type="expression" dxfId="8" priority="1">
-      <formula>AND($AB5&lt;&gt;"yes",$AB5&lt;&gt;"y",$AB5&lt;&gt;"true",$AB5&lt;&gt;"1")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AG5:AG504">
-    <cfRule type="expression" dxfId="9" priority="1">
-      <formula>AND($AB5&lt;&gt;"yes",$AB5&lt;&gt;"y",$AB5&lt;&gt;"true",$AB5&lt;&gt;"1")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AI5:AI504">
-    <cfRule type="expression" dxfId="10" priority="1">
-      <formula>AND($AB5&lt;&gt;"yes",$AB5&lt;&gt;"y",$AB5&lt;&gt;"true",$AB5&lt;&gt;"1")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AJ5:AJ504">
-    <cfRule type="expression" dxfId="11" priority="1">
-      <formula>AND($AB5&lt;&gt;"yes",$AB5&lt;&gt;"y",$AB5&lt;&gt;"true",$AB5&lt;&gt;"1")</formula>
-    </cfRule>
-  </conditionalFormatting>
   <dataValidations count="7">
     <dataValidation type="list" showErrorMessage="1" errorStyle="warning" errorTitle="Invalid value" error="Allowed: personal, company" sqref="A4:A504">
       <formula1>"personal,company"</formula1>

</xml_diff>